<commit_message>
feat(pricing): image pipeline, bailian cache policy, and governance refresh
Add image upstream/compare Excel flow aligned with text, including AIGC tier
mapping fixes and ≥50% supplier deviation review flags. Implement per-model
Bailian Context Cache ratios and regenerate supplier outputs. Sync official
pricing skill, seeds, validators, and W26/W27 weekly notes.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/pricing/output/trinity-pricing-text.xlsx
+++ b/pricing/output/trinity-pricing-text.xlsx
@@ -3166,34 +3166,34 @@
         <v>—</v>
       </c>
       <c r="H52" t="str">
-        <v>入 ¥2.1 · 出 ¥8.4 · 缓 ¥0.42</v>
+        <v>入 ¥4.2 · 出 ¥16.8 · 缓 ¥0.84</v>
       </c>
       <c r="I52" t="str">
         <v>入 $0.3 · 出 $1.2 · 缓 $0.06</v>
       </c>
       <c r="J52" t="str">
-        <v>入 $0.323077 · 出 $1.292308 · 缓 $0.064615</v>
+        <v>入 $0.646154 · 出 $2.584615 · 缓 $0.129231</v>
       </c>
       <c r="K52" t="str">
-        <v>0%</v>
+        <v>+100%</v>
       </c>
       <c r="L52" t="str">
-        <v>0%</v>
+        <v>+100%</v>
       </c>
       <c r="M52" t="str">
-        <v>0%</v>
+        <v>+100%</v>
       </c>
       <c r="N52" t="str">
         <v>—</v>
       </c>
       <c r="O52" t="str">
-        <v>入✅ 出✅ 缓✅</v>
+        <v>入⚠+100% 出⚠+100% 缓⚠+100%</v>
       </c>
       <c r="P52" t="str">
         <v>入⚠-7.1% 出⚠-7.1% 缓⚠-7.1%</v>
       </c>
       <c r="Q52" t="str">
-        <v>入✅ 出✅ 缓✅</v>
+        <v>入⚠+100% 出⚠+100% 缓⚠+100%</v>
       </c>
       <c r="R52" t="str">
         <v>512k 以上输入档仍在内测开放中</v>
@@ -6262,7 +6262,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:K29"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6307,31 +6307,31 @@
         <v>23</v>
       </c>
       <c r="C2">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
       <c r="F2">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G2">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="H2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I2" t="str">
-        <v>+900% ~ +3900%</v>
+        <v>+100% ~ +3900%</v>
       </c>
       <c r="J2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K2" t="str">
-        <v>deepseek-v4-flash(+900%)；deepseek-v4-pro(+3900%)</v>
+        <v>deepseek-v4-flash(+900%)；deepseek-v4-pro(+3900%)；minimax-m3(+100%)</v>
       </c>
     </row>
     <row r="3">
@@ -6517,31 +6517,31 @@
         <v>56</v>
       </c>
       <c r="C8">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8">
         <v>0</v>
       </c>
       <c r="F8">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G8">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="H8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I8" t="str">
-        <v>—</v>
+        <v>+100%</v>
       </c>
       <c r="J8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K8" t="str">
-        <v>—</v>
+        <v>minimax-m3(+100%)</v>
       </c>
     </row>
     <row r="10">
@@ -6611,22 +6611,22 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>百炼北京</v>
+        <v>TokenHub广州</v>
       </c>
       <c r="B14" t="str">
-        <v>deepseek-v4-flash</v>
+        <v>minimax-m3</v>
       </c>
       <c r="C14" t="str">
-        <v>DeepSeek V4 Flash Direct</v>
+        <v>MiniMax M3</v>
       </c>
       <c r="D14" t="str">
-        <v>统一价</v>
+        <v>512k&lt;输入</v>
       </c>
       <c r="E14" t="str">
-        <v>+900%</v>
+        <v>+100%</v>
       </c>
       <c r="F14" t="str">
-        <v>⚠ 缓+900%</v>
+        <v>⚠ 入+100% 出+100% 缓+100%</v>
       </c>
     </row>
     <row r="15">
@@ -6634,19 +6634,19 @@
         <v>百炼北京</v>
       </c>
       <c r="B15" t="str">
-        <v>deepseek-v4-pro</v>
+        <v>deepseek-v4-flash</v>
       </c>
       <c r="C15" t="str">
-        <v>DeepSeek V4 Pro Direct</v>
+        <v>DeepSeek V4 Flash Direct</v>
       </c>
       <c r="D15" t="str">
         <v>统一价</v>
       </c>
       <c r="E15" t="str">
-        <v>+9500%</v>
+        <v>+900%</v>
       </c>
       <c r="F15" t="str">
-        <v>⚠ 入+300% 出+300% 缓+9500%</v>
+        <v>⚠ 缓+900%</v>
       </c>
     </row>
     <row r="16">
@@ -6654,33 +6654,33 @@
         <v>百炼北京</v>
       </c>
       <c r="B16" t="str">
-        <v>qwen3.5-flash</v>
+        <v>deepseek-v4-pro</v>
       </c>
       <c r="C16" t="str">
-        <v>Qwen3.5 Flash</v>
+        <v>DeepSeek V4 Pro Direct</v>
       </c>
       <c r="D16" t="str">
-        <v>0&lt;输入&lt;=128k</v>
+        <v>统一价</v>
       </c>
       <c r="E16" t="str">
-        <v>+100%</v>
+        <v>+9500%</v>
       </c>
       <c r="F16" t="str">
-        <v>⚠ 缓+100%</v>
+        <v>⚠ 入+300% 出+300% 缓+9500%</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v/>
+        <v>百炼北京</v>
       </c>
       <c r="B17" t="str">
-        <v/>
+        <v>qwen3.5-flash</v>
       </c>
       <c r="C17" t="str">
-        <v/>
+        <v>Qwen3.5 Flash</v>
       </c>
       <c r="D17" t="str">
-        <v>128k&lt;输入&lt;=256k</v>
+        <v>0&lt;输入&lt;=128k</v>
       </c>
       <c r="E17" t="str">
         <v>+100%</v>
@@ -6700,7 +6700,7 @@
         <v/>
       </c>
       <c r="D18" t="str">
-        <v>256k&lt;输入&lt;=1M</v>
+        <v>128k&lt;输入&lt;=256k</v>
       </c>
       <c r="E18" t="str">
         <v>+100%</v>
@@ -6711,16 +6711,16 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>百炼北京</v>
+        <v/>
       </c>
       <c r="B19" t="str">
-        <v>qwen3.5-plus</v>
+        <v/>
       </c>
       <c r="C19" t="str">
-        <v>Qwen3.5 Plus</v>
+        <v/>
       </c>
       <c r="D19" t="str">
-        <v>输入&lt;=128k</v>
+        <v>256k&lt;输入&lt;=1M</v>
       </c>
       <c r="E19" t="str">
         <v>+100%</v>
@@ -6731,16 +6731,16 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v/>
+        <v>百炼北京</v>
       </c>
       <c r="B20" t="str">
-        <v/>
+        <v>qwen3.5-plus</v>
       </c>
       <c r="C20" t="str">
-        <v/>
+        <v>Qwen3.5 Plus</v>
       </c>
       <c r="D20" t="str">
-        <v>128k&lt;输入&lt;=256k</v>
+        <v>输入&lt;=128k</v>
       </c>
       <c r="E20" t="str">
         <v>+100%</v>
@@ -6760,7 +6760,7 @@
         <v/>
       </c>
       <c r="D21" t="str">
-        <v>256k&lt;输入&lt;=1M</v>
+        <v>128k&lt;输入&lt;=256k</v>
       </c>
       <c r="E21" t="str">
         <v>+100%</v>
@@ -6771,22 +6771,22 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>火山方舟</v>
+        <v/>
       </c>
       <c r="B22" t="str">
-        <v>deepseek-v3.2</v>
+        <v/>
       </c>
       <c r="C22" t="str">
-        <v>DeepSeek V3.2</v>
+        <v/>
       </c>
       <c r="D22" t="str">
-        <v>输入(32k,128k]</v>
+        <v>256k&lt;输入&lt;=1M</v>
       </c>
       <c r="E22" t="str">
         <v>+100%</v>
       </c>
       <c r="F22" t="str">
-        <v>⚠ 入+100% 出+100%</v>
+        <v>⚠ 缓+100%</v>
       </c>
     </row>
     <row r="23">
@@ -6794,19 +6794,19 @@
         <v>火山方舟</v>
       </c>
       <c r="B23" t="str">
-        <v>deepseek-v4-flash</v>
+        <v>deepseek-v3.2</v>
       </c>
       <c r="C23" t="str">
-        <v>DeepSeek V4 Flash Direct</v>
+        <v>DeepSeek V3.2</v>
       </c>
       <c r="D23" t="str">
-        <v>统一价</v>
+        <v>输入(32k,128k]</v>
       </c>
       <c r="E23" t="str">
-        <v>+900%</v>
+        <v>+100%</v>
       </c>
       <c r="F23" t="str">
-        <v>⚠ 缓+900%</v>
+        <v>⚠ 入+100% 出+100%</v>
       </c>
     </row>
     <row r="24">
@@ -6814,41 +6814,81 @@
         <v>火山方舟</v>
       </c>
       <c r="B24" t="str">
-        <v>deepseek-v4-pro</v>
+        <v>deepseek-v4-flash</v>
       </c>
       <c r="C24" t="str">
-        <v>DeepSeek V4 Pro Direct</v>
+        <v>DeepSeek V4 Flash Direct</v>
       </c>
       <c r="D24" t="str">
         <v>统一价</v>
       </c>
       <c r="E24" t="str">
+        <v>+900%</v>
+      </c>
+      <c r="F24" t="str">
+        <v>⚠ 缓+900%</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>火山方舟</v>
+      </c>
+      <c r="B25" t="str">
+        <v>deepseek-v4-pro</v>
+      </c>
+      <c r="C25" t="str">
+        <v>DeepSeek V4 Pro Direct</v>
+      </c>
+      <c r="D25" t="str">
+        <v>统一价</v>
+      </c>
+      <c r="E25" t="str">
         <v>+3900%</v>
       </c>
-      <c r="F24" t="str">
+      <c r="F25" t="str">
         <v>⚠ 入+300% 出+300% 缓+3900%</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>生成时间：2026-07-03T07:41:47Z</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="str">
+        <v>中转站-cust</v>
+      </c>
+      <c r="B26" t="str">
+        <v>minimax-m3</v>
+      </c>
+      <c r="C26" t="str">
+        <v>MiniMax M3</v>
+      </c>
+      <c r="D26" t="str">
+        <v>512k&lt;输入</v>
+      </c>
+      <c r="E26" t="str">
+        <v>+100%</v>
+      </c>
+      <c r="F26" t="str">
+        <v>⚠ 入+100% 出+100% 缓+100%</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>生成时间：2026-07-03T09:37:10Z</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
         <v>说明：一致=与厂商官方价偏差&lt;0.5%（含 FX 7.5/7.25/6.5 最佳匹配）；不一致上浮=供应商高于官方的偏差%；模型级不一致=任一档位不一致</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K27"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K29"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K35"/>
+  <dimension ref="A1:K34"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -7755,7 +7795,7 @@
         <v>MiniMax</v>
       </c>
       <c r="E28" t="str">
-        <v>输入&lt;=512k</v>
+        <v>512k&lt;输入</v>
       </c>
       <c r="F28" t="str">
         <v>minimax-m3</v>
@@ -7764,10 +7804,10 @@
         <v>入 ¥2.1 · 出 ¥8.4 · 缓 ¥0.42</v>
       </c>
       <c r="H28" t="str">
-        <v>入 ¥2.1 · 出 ¥8.4 · 缓 ¥0.42</v>
+        <v>入 ¥4.2 · 出 ¥16.8 · 缓 ¥0.84</v>
       </c>
       <c r="I28" t="str">
-        <v>✅ 一致</v>
+        <v>⚠ 入+100% 出+100% 缓+100%</v>
       </c>
       <c r="J28" t="str">
         <v>待填</v>
@@ -7780,17 +7820,26 @@
       <c r="A29">
         <v>28</v>
       </c>
+      <c r="B29" t="str">
+        <v>qwen3.5-flash</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Qwen3.5 Flash</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Tongyi</v>
+      </c>
       <c r="E29" t="str">
-        <v>512k&lt;输入</v>
+        <v>0&lt;输入&lt;=128k</v>
       </c>
       <c r="F29" t="str">
-        <v>minimax-m3</v>
+        <v>qwen3.5-flash</v>
       </c>
       <c r="G29" t="str">
-        <v>入 ¥4.2 · 出 ¥16.8 · 缓 ¥0.84</v>
+        <v>入 ¥0.2 · 出 ¥2 · 缓 ¥0.02</v>
       </c>
       <c r="H29" t="str">
-        <v>入 ¥4.2 · 出 ¥16.8 · 缓 ¥0.84</v>
+        <v>入 ¥0.2 · 出 ¥2 · 缓 ¥0.02</v>
       </c>
       <c r="I29" t="str">
         <v>✅ 一致</v>
@@ -7806,26 +7855,17 @@
       <c r="A30">
         <v>29</v>
       </c>
-      <c r="B30" t="str">
-        <v>qwen3.5-flash</v>
-      </c>
-      <c r="C30" t="str">
-        <v>Qwen3.5 Flash</v>
-      </c>
-      <c r="D30" t="str">
-        <v>Tongyi</v>
-      </c>
       <c r="E30" t="str">
-        <v>0&lt;输入&lt;=128k</v>
+        <v>128k&lt;输入&lt;=256k</v>
       </c>
       <c r="F30" t="str">
         <v>qwen3.5-flash</v>
       </c>
       <c r="G30" t="str">
-        <v>入 ¥0.2 · 出 ¥2 · 缓 ¥0.02</v>
+        <v>入 ¥0.8 · 出 ¥8 · 缓 ¥0.08</v>
       </c>
       <c r="H30" t="str">
-        <v>入 ¥0.2 · 出 ¥2 · 缓 ¥0.02</v>
+        <v>入 ¥0.8 · 出 ¥8 · 缓 ¥0.08</v>
       </c>
       <c r="I30" t="str">
         <v>✅ 一致</v>
@@ -7842,16 +7882,16 @@
         <v>30</v>
       </c>
       <c r="E31" t="str">
-        <v>128k&lt;输入&lt;=256k</v>
+        <v>256k&lt;输入&lt;=1M</v>
       </c>
       <c r="F31" t="str">
         <v>qwen3.5-flash</v>
       </c>
       <c r="G31" t="str">
-        <v>入 ¥0.8 · 出 ¥8 · 缓 ¥0.08</v>
+        <v>入 ¥1.2 · 出 ¥12 · 缓 ¥0.12</v>
       </c>
       <c r="H31" t="str">
-        <v>入 ¥0.8 · 出 ¥8 · 缓 ¥0.08</v>
+        <v>入 ¥1.2 · 出 ¥12 · 缓 ¥0.12</v>
       </c>
       <c r="I31" t="str">
         <v>✅ 一致</v>
@@ -7867,17 +7907,26 @@
       <c r="A32">
         <v>31</v>
       </c>
+      <c r="B32" t="str">
+        <v>qwen3.5-plus</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Qwen3.5 Plus</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Tongyi</v>
+      </c>
       <c r="E32" t="str">
-        <v>256k&lt;输入&lt;=1M</v>
+        <v>输入&lt;=128k</v>
       </c>
       <c r="F32" t="str">
-        <v>qwen3.5-flash</v>
+        <v>qwen3.5-plus</v>
       </c>
       <c r="G32" t="str">
-        <v>入 ¥1.2 · 出 ¥12 · 缓 ¥0.12</v>
+        <v>入 ¥0.8 · 出 ¥4.8 · 缓 ¥0.08</v>
       </c>
       <c r="H32" t="str">
-        <v>入 ¥1.2 · 出 ¥12 · 缓 ¥0.12</v>
+        <v>入 ¥0.8 · 出 ¥4.8 · 缓 ¥0.08</v>
       </c>
       <c r="I32" t="str">
         <v>✅ 一致</v>
@@ -7893,26 +7942,17 @@
       <c r="A33">
         <v>32</v>
       </c>
-      <c r="B33" t="str">
-        <v>qwen3.5-plus</v>
-      </c>
-      <c r="C33" t="str">
-        <v>Qwen3.5 Plus</v>
-      </c>
-      <c r="D33" t="str">
-        <v>Tongyi</v>
-      </c>
       <c r="E33" t="str">
-        <v>输入&lt;=128k</v>
+        <v>128k&lt;输入&lt;=256k</v>
       </c>
       <c r="F33" t="str">
         <v>qwen3.5-plus</v>
       </c>
       <c r="G33" t="str">
-        <v>入 ¥0.8 · 出 ¥4.8 · 缓 ¥0.08</v>
+        <v>入 ¥2 · 出 ¥12 · 缓 ¥0.2</v>
       </c>
       <c r="H33" t="str">
-        <v>入 ¥0.8 · 出 ¥4.8 · 缓 ¥0.08</v>
+        <v>入 ¥2 · 出 ¥12 · 缓 ¥0.2</v>
       </c>
       <c r="I33" t="str">
         <v>✅ 一致</v>
@@ -7929,16 +7969,16 @@
         <v>33</v>
       </c>
       <c r="E34" t="str">
-        <v>128k&lt;输入&lt;=256k</v>
+        <v>256k&lt;输入&lt;=1M</v>
       </c>
       <c r="F34" t="str">
         <v>qwen3.5-plus</v>
       </c>
       <c r="G34" t="str">
-        <v>入 ¥2 · 出 ¥12 · 缓 ¥0.2</v>
+        <v>入 ¥4 · 出 ¥24 · 缓 ¥0.4</v>
       </c>
       <c r="H34" t="str">
-        <v>入 ¥2 · 出 ¥12 · 缓 ¥0.2</v>
+        <v>入 ¥4 · 出 ¥24 · 缓 ¥0.4</v>
       </c>
       <c r="I34" t="str">
         <v>✅ 一致</v>
@@ -7950,34 +7990,8 @@
         <v>待填</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35">
-        <v>34</v>
-      </c>
-      <c r="E35" t="str">
-        <v>256k&lt;输入&lt;=1M</v>
-      </c>
-      <c r="F35" t="str">
-        <v>qwen3.5-plus</v>
-      </c>
-      <c r="G35" t="str">
-        <v>入 ¥4 · 出 ¥24 · 缓 ¥0.4</v>
-      </c>
-      <c r="H35" t="str">
-        <v>入 ¥4 · 出 ¥24 · 缓 ¥0.4</v>
-      </c>
-      <c r="I35" t="str">
-        <v>✅ 一致</v>
-      </c>
-      <c r="J35" t="str">
-        <v>待填</v>
-      </c>
-      <c r="K35" t="str">
-        <v>待填</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="24">
+  <mergeCells count="21">
     <mergeCell ref="B5:B6"/>
     <mergeCell ref="C5:C6"/>
     <mergeCell ref="D5:D6"/>
@@ -7993,18 +8007,15 @@
     <mergeCell ref="B19:B21"/>
     <mergeCell ref="C19:C21"/>
     <mergeCell ref="D19:D21"/>
-    <mergeCell ref="B28:B29"/>
-    <mergeCell ref="C28:C29"/>
-    <mergeCell ref="D28:D29"/>
-    <mergeCell ref="B30:B32"/>
-    <mergeCell ref="C30:C32"/>
-    <mergeCell ref="D30:D32"/>
-    <mergeCell ref="B33:B35"/>
-    <mergeCell ref="C33:C35"/>
-    <mergeCell ref="D33:D35"/>
+    <mergeCell ref="B29:B31"/>
+    <mergeCell ref="C29:C31"/>
+    <mergeCell ref="D29:D31"/>
+    <mergeCell ref="B32:B34"/>
+    <mergeCell ref="C32:C34"/>
+    <mergeCell ref="D32:D34"/>
   </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K34"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -16774,13 +16785,13 @@
         <v>minimax-m3</v>
       </c>
       <c r="G54" t="str">
-        <v>入 ¥4.2 · 出 ¥16.8 · 缓 ¥0.84</v>
+        <v>入 ¥2.1 · 出 ¥8.4 · 缓 ¥0.42</v>
       </c>
       <c r="H54" t="str">
         <v>入 ¥4.2 · 出 ¥16.8 · 缓 ¥0.84</v>
       </c>
       <c r="I54" t="str">
-        <v>✅ 一致</v>
+        <v>⚠ 入+100% 出+100% 缓+100%</v>
       </c>
       <c r="J54" t="str">
         <v>—</v>

</xml_diff>